<commit_message>
Add option module rule: 'o' on BLENDING/RECIRCULATION/SRU/FEED PUMP → False/False
Updated Excel adds dedicated Option column (col D); BREW 350/450 shifted to E/F.
parse_excel now detects the Option column header and builds option_tags set.
xlval_to_enable_exist and has_fb accept is_option flag: 'o' for option-type
instruments resolves to ENABLE=False, EXIST=False, VLV_W_FB=False.
Result: OK count per family improved from 58 to 64. Verification passed.
Updated wishList.md, DesignStructure.md, PROJECT_LEARNINGS.md accordingly.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/InstrumentStatusComparison.xlsx
+++ b/InstrumentStatusComparison.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3047" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3047" uniqueCount="296">
   <si>
     <t>TIA Portal DB Instrument Status Comparison Report</t>
   </si>
@@ -111,277 +111,280 @@
     <t>DIFF</t>
   </si>
   <si>
+    <t>UPDATE: VLV_W_FB: DB=True-&gt;False</t>
+  </si>
+  <si>
+    <t>AV210-1</t>
+  </si>
+  <si>
+    <t>EM - 210</t>
+  </si>
+  <si>
+    <t>UPDATE: EXIST: DB=True-&gt;False, VLV_W_FB: DB=True-&gt;False</t>
+  </si>
+  <si>
+    <t>AV212-1</t>
+  </si>
+  <si>
+    <t>EM - 212</t>
+  </si>
+  <si>
+    <t>AV220-1</t>
+  </si>
+  <si>
+    <t>EM - 22X</t>
+  </si>
+  <si>
+    <t>AV221-1</t>
+  </si>
+  <si>
+    <t>EM - 22Y</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>AV222-1</t>
+  </si>
+  <si>
+    <t>Unit Dch</t>
+  </si>
+  <si>
+    <t>EM - 222</t>
+  </si>
+  <si>
+    <t>AV301-1</t>
+  </si>
+  <si>
+    <t>EM - 300</t>
+  </si>
+  <si>
+    <t>AV320-1</t>
+  </si>
+  <si>
+    <t>AV340-1</t>
+  </si>
+  <si>
+    <t>EM - 340</t>
+  </si>
+  <si>
+    <t>AV340-2</t>
+  </si>
+  <si>
+    <t>AV460-1</t>
+  </si>
+  <si>
+    <t>AV460-2</t>
+  </si>
+  <si>
+    <t>AV460d-1</t>
+  </si>
+  <si>
+    <t>Unit Sep</t>
+  </si>
+  <si>
+    <t>EM - 460</t>
+  </si>
+  <si>
+    <t>AV543-1</t>
+  </si>
+  <si>
+    <t>EM - 506</t>
+  </si>
+  <si>
+    <t>AV463-1</t>
+  </si>
+  <si>
+    <t>EM - 463</t>
+  </si>
+  <si>
+    <t>UPDATE: ENABLE: DB=False-&gt;True, EXIST: DB=True-&gt;False</t>
+  </si>
+  <si>
+    <t>AV463-2</t>
+  </si>
+  <si>
+    <t>AV461-1</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>NOT IN TAG_MAP</t>
+  </si>
+  <si>
+    <t>FIS409-1</t>
+  </si>
+  <si>
+    <t>COOLING LIQUID FLOW</t>
+  </si>
+  <si>
+    <t>EM - 400</t>
+  </si>
+  <si>
+    <t>FIS615-1</t>
+  </si>
+  <si>
+    <t>SEALING LIQUID FLOW INLET SEAL</t>
+  </si>
+  <si>
+    <t>EM - 600</t>
+  </si>
+  <si>
+    <t>FIS635-1</t>
+  </si>
+  <si>
+    <t>SEALING LIQUID FLOW OUTLET SEAL</t>
+  </si>
+  <si>
+    <t>FIS630-1</t>
+  </si>
+  <si>
+    <t>UPDATE: EXIST: DB=True-&gt;False</t>
+  </si>
+  <si>
+    <t>PIS340-1</t>
+  </si>
+  <si>
+    <t>SAFETY LIQUID PRESSURE</t>
+  </si>
+  <si>
+    <t>PIS375-1</t>
+  </si>
+  <si>
+    <t>OP. LIQUID PRESSURE</t>
+  </si>
+  <si>
+    <t>EM - 375</t>
+  </si>
+  <si>
+    <t>PS502-1</t>
+  </si>
+  <si>
+    <t>INSTRUMENT AIR PRESSURE</t>
+  </si>
+  <si>
+    <t>EM - 100</t>
+  </si>
+  <si>
+    <t>QT201-1_OK</t>
+  </si>
+  <si>
+    <t>HEALTHY STATUS</t>
+  </si>
+  <si>
+    <t>QT220-1_OK</t>
+  </si>
+  <si>
+    <t>QT220-2_OK</t>
+  </si>
+  <si>
+    <t>NOT FOUND IN DB</t>
+  </si>
+  <si>
+    <t>eWON</t>
+  </si>
+  <si>
+    <t>eWON Talk2M STATUS</t>
+  </si>
+  <si>
+    <t>UPDATE: ENABLE: DB=False-&gt;True, EXIST: DB=False-&gt;True</t>
+  </si>
+  <si>
+    <t>LA201-1</t>
+  </si>
+  <si>
+    <t>INLET SIGHT GLASS BACKLIGHT</t>
+  </si>
+  <si>
+    <t>LA220-1</t>
+  </si>
+  <si>
+    <t>OUTLET SIGHT GLASS BACKLIGHT</t>
+  </si>
+  <si>
+    <t>L-GN</t>
+  </si>
+  <si>
+    <t>SIGNAL TOWER-GREEN LIGHT</t>
+  </si>
+  <si>
+    <t>L-YL</t>
+  </si>
+  <si>
+    <t>SIGNAL TOWER-YELLOW LIGHT</t>
+  </si>
+  <si>
+    <t>L-RD</t>
+  </si>
+  <si>
+    <t>SIGNAL TOWER-RED LIGHT/ALARM LIGHT</t>
+  </si>
+  <si>
+    <t>L-BUZZ</t>
+  </si>
+  <si>
+    <t>SIGNAL TOWER-BUZZIER</t>
+  </si>
+  <si>
+    <t>LA221-1</t>
+  </si>
+  <si>
+    <t>PIT201-1</t>
+  </si>
+  <si>
+    <t>INLET PRESSURE</t>
+  </si>
+  <si>
+    <t>PIT22X-1</t>
+  </si>
+  <si>
+    <t>SEPARATOR OUTLET 220 PRESSURE</t>
+  </si>
+  <si>
+    <t>QT201-1</t>
+  </si>
+  <si>
+    <t>INLET TURBIDITY</t>
+  </si>
+  <si>
+    <t>QT220-1</t>
+  </si>
+  <si>
+    <t>OUTLET TURBIDITY</t>
+  </si>
+  <si>
+    <t>QT220-2</t>
+  </si>
+  <si>
+    <t>PIT22Y-1</t>
+  </si>
+  <si>
+    <t>SEPARATOR OUTLET 221 PRESSURE</t>
+  </si>
+  <si>
+    <t>PIT222-1</t>
+  </si>
+  <si>
+    <t>SOLIDS OUTLET PRESSURE</t>
+  </si>
+  <si>
+    <t>LT-BT</t>
+  </si>
+  <si>
+    <t>BUFFER TANK LEVEL</t>
+  </si>
+  <si>
+    <t>N/F</t>
+  </si>
+  <si>
+    <t>LT463-1</t>
+  </si>
+  <si>
+    <t>LEVEL IN B463-1</t>
+  </si>
+  <si>
     <t>UPDATE: ENABLE: DB=False-&gt;True</t>
-  </si>
-  <si>
-    <t>AV210-1</t>
-  </si>
-  <si>
-    <t>EM - 210</t>
-  </si>
-  <si>
-    <t>UPDATE: ENABLE: DB=False-&gt;True, EXIST: DB=True-&gt;False</t>
-  </si>
-  <si>
-    <t>AV212-1</t>
-  </si>
-  <si>
-    <t>EM - 212</t>
-  </si>
-  <si>
-    <t>AV220-1</t>
-  </si>
-  <si>
-    <t>EM - 22X</t>
-  </si>
-  <si>
-    <t>AV221-1</t>
-  </si>
-  <si>
-    <t>EM - 22Y</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>UPDATE: EXIST: DB=True-&gt;False, VLV_W_FB: DB=True-&gt;False</t>
-  </si>
-  <si>
-    <t>AV222-1</t>
-  </si>
-  <si>
-    <t>Unit Dch</t>
-  </si>
-  <si>
-    <t>EM - 222</t>
-  </si>
-  <si>
-    <t>AV301-1</t>
-  </si>
-  <si>
-    <t>EM - 300</t>
-  </si>
-  <si>
-    <t>AV320-1</t>
-  </si>
-  <si>
-    <t>AV340-1</t>
-  </si>
-  <si>
-    <t>EM - 340</t>
-  </si>
-  <si>
-    <t>AV340-2</t>
-  </si>
-  <si>
-    <t>AV460-1</t>
-  </si>
-  <si>
-    <t>AV460-2</t>
-  </si>
-  <si>
-    <t>AV460d-1</t>
-  </si>
-  <si>
-    <t>Unit Sep</t>
-  </si>
-  <si>
-    <t>EM - 460</t>
-  </si>
-  <si>
-    <t>AV543-1</t>
-  </si>
-  <si>
-    <t>EM - 506</t>
-  </si>
-  <si>
-    <t>AV463-1</t>
-  </si>
-  <si>
-    <t>EM - 463</t>
-  </si>
-  <si>
-    <t>AV463-2</t>
-  </si>
-  <si>
-    <t>AV461-1</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>NOT IN TAG_MAP</t>
-  </si>
-  <si>
-    <t>FIS409-1</t>
-  </si>
-  <si>
-    <t>COOLING LIQUID FLOW</t>
-  </si>
-  <si>
-    <t>EM - 400</t>
-  </si>
-  <si>
-    <t>FIS615-1</t>
-  </si>
-  <si>
-    <t>SEALING LIQUID FLOW INLET SEAL</t>
-  </si>
-  <si>
-    <t>EM - 600</t>
-  </si>
-  <si>
-    <t>FIS635-1</t>
-  </si>
-  <si>
-    <t>SEALING LIQUID FLOW OUTLET SEAL</t>
-  </si>
-  <si>
-    <t>FIS630-1</t>
-  </si>
-  <si>
-    <t>UPDATE: EXIST: DB=True-&gt;False</t>
-  </si>
-  <si>
-    <t>PIS340-1</t>
-  </si>
-  <si>
-    <t>SAFETY LIQUID PRESSURE</t>
-  </si>
-  <si>
-    <t>PIS375-1</t>
-  </si>
-  <si>
-    <t>OP. LIQUID PRESSURE</t>
-  </si>
-  <si>
-    <t>EM - 375</t>
-  </si>
-  <si>
-    <t>PS502-1</t>
-  </si>
-  <si>
-    <t>INSTRUMENT AIR PRESSURE</t>
-  </si>
-  <si>
-    <t>EM - 100</t>
-  </si>
-  <si>
-    <t>QT201-1_OK</t>
-  </si>
-  <si>
-    <t>HEALTHY STATUS</t>
-  </si>
-  <si>
-    <t>QT220-1_OK</t>
-  </si>
-  <si>
-    <t>QT220-2_OK</t>
-  </si>
-  <si>
-    <t>N/F</t>
-  </si>
-  <si>
-    <t>NOT FOUND IN DB</t>
-  </si>
-  <si>
-    <t>eWON</t>
-  </si>
-  <si>
-    <t>eWON Talk2M STATUS</t>
-  </si>
-  <si>
-    <t>UPDATE: ENABLE: DB=False-&gt;True, EXIST: DB=False-&gt;True</t>
-  </si>
-  <si>
-    <t>LA201-1</t>
-  </si>
-  <si>
-    <t>INLET SIGHT GLASS BACKLIGHT</t>
-  </si>
-  <si>
-    <t>LA220-1</t>
-  </si>
-  <si>
-    <t>OUTLET SIGHT GLASS BACKLIGHT</t>
-  </si>
-  <si>
-    <t>L-GN</t>
-  </si>
-  <si>
-    <t>SIGNAL TOWER-GREEN LIGHT</t>
-  </si>
-  <si>
-    <t>L-YL</t>
-  </si>
-  <si>
-    <t>SIGNAL TOWER-YELLOW LIGHT</t>
-  </si>
-  <si>
-    <t>L-RD</t>
-  </si>
-  <si>
-    <t>SIGNAL TOWER-RED LIGHT/ALARM LIGHT</t>
-  </si>
-  <si>
-    <t>L-BUZZ</t>
-  </si>
-  <si>
-    <t>SIGNAL TOWER-BUZZIER</t>
-  </si>
-  <si>
-    <t>LA221-1</t>
-  </si>
-  <si>
-    <t>PIT201-1</t>
-  </si>
-  <si>
-    <t>INLET PRESSURE</t>
-  </si>
-  <si>
-    <t>PIT22X-1</t>
-  </si>
-  <si>
-    <t>SEPARATOR OUTLET 220 PRESSURE</t>
-  </si>
-  <si>
-    <t>QT201-1</t>
-  </si>
-  <si>
-    <t>INLET TURBIDITY</t>
-  </si>
-  <si>
-    <t>QT220-1</t>
-  </si>
-  <si>
-    <t>OUTLET TURBIDITY</t>
-  </si>
-  <si>
-    <t>QT220-2</t>
-  </si>
-  <si>
-    <t>PIT22Y-1</t>
-  </si>
-  <si>
-    <t>SEPARATOR OUTLET 221 PRESSURE</t>
-  </si>
-  <si>
-    <t>PIT222-1</t>
-  </si>
-  <si>
-    <t>SOLIDS OUTLET PRESSURE</t>
-  </si>
-  <si>
-    <t>LT-BT</t>
-  </si>
-  <si>
-    <t>BUFFER TANK LEVEL</t>
-  </si>
-  <si>
-    <t>LT463-1</t>
-  </si>
-  <si>
-    <t>LEVEL IN B463-1</t>
   </si>
   <si>
     <t>PIT463-1</t>
@@ -1549,14 +1552,14 @@
       <c r="E5" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F5" s="5" t="s">
-        <v>21</v>
+      <c r="F5" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>27</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>27</v>
@@ -1576,14 +1579,14 @@
       <c r="N5" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="O5" s="5" t="s">
-        <v>21</v>
+      <c r="O5" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="P5" s="4" t="s">
         <v>27</v>
       </c>
       <c r="Q5" s="4" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="R5" s="4" t="s">
         <v>27</v>
@@ -1617,14 +1620,14 @@
       <c r="E6" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F6" s="5" t="s">
-        <v>21</v>
+      <c r="F6" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>27</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I6" s="4" t="s">
         <v>27</v>
@@ -1644,14 +1647,14 @@
       <c r="N6" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="O6" s="5" t="s">
-        <v>21</v>
+      <c r="O6" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="P6" s="4" t="s">
         <v>27</v>
       </c>
       <c r="Q6" s="4" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="R6" s="4" t="s">
         <v>27</v>
@@ -1843,7 +1846,7 @@
         <v>28</v>
       </c>
       <c r="M9" s="7" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="N9" s="4" t="s">
         <v>39</v>
@@ -1870,21 +1873,21 @@
         <v>28</v>
       </c>
       <c r="V9" s="7" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:22">
       <c r="A10" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>17</v>
       </c>
       <c r="C10" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>42</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>43</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>20</v>
@@ -1943,16 +1946,16 @@
     </row>
     <row r="11" spans="1:22">
       <c r="A11" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>17</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>20</v>
@@ -2011,16 +2014,16 @@
     </row>
     <row r="12" spans="1:22">
       <c r="A12" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>17</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>20</v>
@@ -2079,7 +2082,7 @@
     </row>
     <row r="13" spans="1:22">
       <c r="A13" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>17</v>
@@ -2088,7 +2091,7 @@
         <v>18</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>20</v>
@@ -2147,7 +2150,7 @@
     </row>
     <row r="14" spans="1:22">
       <c r="A14" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>17</v>
@@ -2156,7 +2159,7 @@
         <v>18</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>20</v>
@@ -2215,7 +2218,7 @@
     </row>
     <row r="15" spans="1:22">
       <c r="A15" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>17</v>
@@ -2283,7 +2286,7 @@
     </row>
     <row r="16" spans="1:22">
       <c r="A16" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>17</v>
@@ -2292,7 +2295,7 @@
         <v>18</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>20</v>
@@ -2351,16 +2354,16 @@
     </row>
     <row r="17" spans="1:22">
       <c r="A17" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>17</v>
       </c>
       <c r="C17" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D17" s="4" t="s">
         <v>53</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>54</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>39</v>
@@ -2387,7 +2390,7 @@
         <v>28</v>
       </c>
       <c r="M17" s="7" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="N17" s="5" t="s">
         <v>20</v>
@@ -2419,16 +2422,16 @@
     </row>
     <row r="18" spans="1:22">
       <c r="A18" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>17</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>20</v>
@@ -2487,7 +2490,7 @@
     </row>
     <row r="19" spans="1:22">
       <c r="A19" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>17</v>
@@ -2496,7 +2499,7 @@
         <v>24</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>39</v>
@@ -2523,7 +2526,7 @@
         <v>28</v>
       </c>
       <c r="M19" s="7" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="N19" s="6" t="s">
         <v>26</v>
@@ -2550,7 +2553,7 @@
         <v>28</v>
       </c>
       <c r="V19" s="7" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
     </row>
     <row r="20" spans="1:22">
@@ -2564,7 +2567,7 @@
         <v>24</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>39</v>
@@ -2591,7 +2594,7 @@
         <v>28</v>
       </c>
       <c r="M20" s="7" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="N20" s="6" t="s">
         <v>26</v>
@@ -2618,7 +2621,7 @@
         <v>28</v>
       </c>
       <c r="V20" s="7" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
     </row>
     <row r="21" spans="1:22">
@@ -2659,7 +2662,7 @@
         <v>28</v>
       </c>
       <c r="M21" s="7" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="N21" s="4" t="s">
         <v>39</v>
@@ -2686,7 +2689,7 @@
         <v>28</v>
       </c>
       <c r="V21" s="7" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
     </row>
     <row r="22" spans="1:22">
@@ -2765,7 +2768,7 @@
         <v>64</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>65</v>
@@ -2833,7 +2836,7 @@
         <v>67</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>68</v>
@@ -2901,7 +2904,7 @@
         <v>70</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>68</v>
@@ -2969,7 +2972,7 @@
         <v>70</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>68</v>
@@ -3040,7 +3043,7 @@
         <v>18</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E27" s="5" t="s">
         <v>20</v>
@@ -3105,7 +3108,7 @@
         <v>76</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>77</v>
@@ -3173,7 +3176,7 @@
         <v>79</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>80</v>
@@ -3385,8 +3388,8 @@
       <c r="E32" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F32" s="5" t="s">
-        <v>21</v>
+      <c r="F32" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="G32" s="4" t="s">
         <v>27</v>
@@ -3403,17 +3406,17 @@
       <c r="K32" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="L32" s="6" t="s">
+      <c r="L32" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="M32" s="6" t="s">
         <v>85</v>
-      </c>
-      <c r="M32" s="6" t="s">
-        <v>86</v>
       </c>
       <c r="N32" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="O32" s="5" t="s">
-        <v>21</v>
+      <c r="O32" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="P32" s="4" t="s">
         <v>27</v>
@@ -3430,22 +3433,22 @@
       <c r="T32" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="U32" s="6" t="s">
+      <c r="U32" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="V32" s="6" t="s">
         <v>85</v>
-      </c>
-      <c r="V32" s="6" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="33" spans="1:22">
       <c r="A33" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B33" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B33" s="4" t="s">
-        <v>88</v>
-      </c>
       <c r="C33" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>80</v>
@@ -3475,7 +3478,7 @@
         <v>28</v>
       </c>
       <c r="M33" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="N33" s="5" t="s">
         <v>20</v>
@@ -3502,15 +3505,15 @@
         <v>28</v>
       </c>
       <c r="V33" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="34" spans="1:22">
       <c r="A34" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B34" s="4" t="s">
         <v>90</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>91</v>
       </c>
       <c r="C34" s="4" t="s">
         <v>18</v>
@@ -3575,10 +3578,10 @@
     </row>
     <row r="35" spans="1:22">
       <c r="A35" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B35" s="4" t="s">
         <v>92</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>93</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>18</v>
@@ -3643,13 +3646,13 @@
     </row>
     <row r="36" spans="1:22">
       <c r="A36" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B36" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="B36" s="4" t="s">
-        <v>95</v>
-      </c>
       <c r="C36" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D36" s="4" t="s">
         <v>80</v>
@@ -3711,13 +3714,13 @@
     </row>
     <row r="37" spans="1:22">
       <c r="A37" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B37" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B37" s="4" t="s">
-        <v>97</v>
-      </c>
       <c r="C37" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>80</v>
@@ -3779,13 +3782,13 @@
     </row>
     <row r="38" spans="1:22">
       <c r="A38" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B38" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B38" s="4" t="s">
-        <v>99</v>
-      </c>
       <c r="C38" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D38" s="4" t="s">
         <v>80</v>
@@ -3847,13 +3850,13 @@
     </row>
     <row r="39" spans="1:22">
       <c r="A39" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B39" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="B39" s="4" t="s">
-        <v>101</v>
-      </c>
       <c r="C39" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D39" s="4" t="s">
         <v>80</v>
@@ -3915,10 +3918,10 @@
     </row>
     <row r="40" spans="1:22">
       <c r="A40" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>18</v>
@@ -3983,10 +3986,10 @@
     </row>
     <row r="41" spans="1:22">
       <c r="A41" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B41" s="4" t="s">
         <v>103</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>18</v>
@@ -4051,10 +4054,10 @@
     </row>
     <row r="42" spans="1:22">
       <c r="A42" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B42" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="B42" s="4" t="s">
-        <v>106</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>18</v>
@@ -4119,10 +4122,10 @@
     </row>
     <row r="43" spans="1:22">
       <c r="A43" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B43" s="4" t="s">
         <v>107</v>
-      </c>
-      <c r="B43" s="4" t="s">
-        <v>108</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>18</v>
@@ -4187,10 +4190,10 @@
     </row>
     <row r="44" spans="1:22">
       <c r="A44" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B44" s="4" t="s">
         <v>109</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>110</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>18</v>
@@ -4255,10 +4258,10 @@
     </row>
     <row r="45" spans="1:22">
       <c r="A45" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C45" s="4" t="s">
         <v>24</v>
@@ -4269,8 +4272,8 @@
       <c r="E45" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F45" s="5" t="s">
-        <v>21</v>
+      <c r="F45" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="G45" s="4" t="s">
         <v>27</v>
@@ -4287,17 +4290,17 @@
       <c r="K45" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="L45" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="M45" s="7" t="s">
-        <v>29</v>
+      <c r="L45" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="M45" s="5" t="s">
+        <v>22</v>
       </c>
       <c r="N45" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="O45" s="5" t="s">
-        <v>21</v>
+      <c r="O45" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="P45" s="4" t="s">
         <v>27</v>
@@ -4314,19 +4317,19 @@
       <c r="T45" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="U45" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="V45" s="7" t="s">
-        <v>29</v>
+      <c r="U45" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="V45" s="5" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="46" spans="1:22">
       <c r="A46" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B46" s="4" t="s">
         <v>112</v>
-      </c>
-      <c r="B46" s="4" t="s">
-        <v>113</v>
       </c>
       <c r="C46" s="4" t="s">
         <v>18</v>
@@ -4391,10 +4394,10 @@
     </row>
     <row r="47" spans="1:22">
       <c r="A47" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B47" s="4" t="s">
         <v>114</v>
-      </c>
-      <c r="B47" s="4" t="s">
-        <v>115</v>
       </c>
       <c r="C47" s="4" t="s">
         <v>61</v>
@@ -4459,13 +4462,13 @@
     </row>
     <row r="48" spans="1:22">
       <c r="A48" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B48" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="B48" s="4" t="s">
-        <v>117</v>
-      </c>
       <c r="C48" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D48" s="4" t="s">
         <v>80</v>
@@ -4492,10 +4495,10 @@
         <v>61</v>
       </c>
       <c r="L48" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="M48" s="6" t="s">
         <v>85</v>
-      </c>
-      <c r="M48" s="6" t="s">
-        <v>86</v>
       </c>
       <c r="N48" s="6" t="s">
         <v>26</v>
@@ -4519,10 +4522,10 @@
         <v>61</v>
       </c>
       <c r="U48" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="V48" s="6" t="s">
         <v>85</v>
-      </c>
-      <c r="V48" s="6" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="49" spans="1:22">
@@ -4536,7 +4539,7 @@
         <v>24</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E49" s="4" t="s">
         <v>39</v>
@@ -4590,21 +4593,21 @@
         <v>28</v>
       </c>
       <c r="V49" s="7" t="s">
-        <v>29</v>
+        <v>120</v>
       </c>
     </row>
     <row r="50" spans="1:22">
       <c r="A50" s="4" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C50" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E50" s="4" t="s">
         <v>39</v>
@@ -4658,27 +4661,27 @@
         <v>28</v>
       </c>
       <c r="V50" s="7" t="s">
-        <v>29</v>
+        <v>120</v>
       </c>
     </row>
     <row r="51" spans="1:22">
       <c r="A51" s="4" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C51" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F51" s="5" t="s">
-        <v>21</v>
+      <c r="F51" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="G51" s="4" t="s">
         <v>27</v>
@@ -4695,17 +4698,17 @@
       <c r="K51" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="L51" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="M51" s="7" t="s">
-        <v>29</v>
+      <c r="L51" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="M51" s="5" t="s">
+        <v>22</v>
       </c>
       <c r="N51" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="O51" s="5" t="s">
-        <v>21</v>
+      <c r="O51" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="P51" s="4" t="s">
         <v>27</v>
@@ -4722,19 +4725,19 @@
       <c r="T51" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="U51" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="V51" s="7" t="s">
-        <v>29</v>
+      <c r="U51" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="V51" s="5" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="52" spans="1:22">
       <c r="A52" s="4" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C52" s="4" t="s">
         <v>18</v>
@@ -4799,10 +4802,10 @@
     </row>
     <row r="53" spans="1:22">
       <c r="A53" s="4" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C53" s="4" t="s">
         <v>24</v>
@@ -4813,8 +4816,8 @@
       <c r="E53" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F53" s="5" t="s">
-        <v>21</v>
+      <c r="F53" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="G53" s="4" t="s">
         <v>27</v>
@@ -4831,17 +4834,17 @@
       <c r="K53" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="L53" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="M53" s="7" t="s">
-        <v>29</v>
+      <c r="L53" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="M53" s="5" t="s">
+        <v>22</v>
       </c>
       <c r="N53" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="O53" s="5" t="s">
-        <v>21</v>
+      <c r="O53" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="P53" s="4" t="s">
         <v>27</v>
@@ -4858,22 +4861,22 @@
       <c r="T53" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="U53" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="V53" s="7" t="s">
-        <v>29</v>
+      <c r="U53" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="V53" s="5" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="54" spans="1:22">
       <c r="A54" s="4" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B54" s="4" t="s">
         <v>64</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D54" s="4" t="s">
         <v>65</v>
@@ -4935,10 +4938,10 @@
     </row>
     <row r="55" spans="1:22">
       <c r="A55" s="4" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C55" s="4" t="s">
         <v>18</v>
@@ -5003,10 +5006,10 @@
     </row>
     <row r="56" spans="1:22">
       <c r="A56" s="4" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C56" s="4" t="s">
         <v>18</v>
@@ -5071,16 +5074,16 @@
     </row>
     <row r="57" spans="1:22">
       <c r="A57" s="4" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E57" s="5" t="s">
         <v>20</v>
@@ -5139,10 +5142,10 @@
     </row>
     <row r="58" spans="1:22">
       <c r="A58" s="4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C58" s="4" t="s">
         <v>18</v>
@@ -5207,10 +5210,10 @@
     </row>
     <row r="59" spans="1:22">
       <c r="A59" s="4" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C59" s="4" t="s">
         <v>24</v>
@@ -5221,8 +5224,8 @@
       <c r="E59" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F59" s="5" t="s">
-        <v>21</v>
+      <c r="F59" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="G59" s="4" t="s">
         <v>27</v>
@@ -5239,17 +5242,17 @@
       <c r="K59" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="L59" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="M59" s="7" t="s">
-        <v>29</v>
+      <c r="L59" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="M59" s="5" t="s">
+        <v>22</v>
       </c>
       <c r="N59" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="O59" s="5" t="s">
-        <v>21</v>
+      <c r="O59" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="P59" s="4" t="s">
         <v>27</v>
@@ -5266,19 +5269,19 @@
       <c r="T59" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="U59" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="V59" s="7" t="s">
-        <v>29</v>
+      <c r="U59" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="V59" s="5" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="60" spans="1:22">
       <c r="A60" s="4" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C60" s="4" t="s">
         <v>24</v>
@@ -5289,8 +5292,8 @@
       <c r="E60" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F60" s="5" t="s">
-        <v>21</v>
+      <c r="F60" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="G60" s="4" t="s">
         <v>27</v>
@@ -5307,17 +5310,17 @@
       <c r="K60" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="L60" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="M60" s="7" t="s">
-        <v>29</v>
+      <c r="L60" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="M60" s="5" t="s">
+        <v>22</v>
       </c>
       <c r="N60" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="O60" s="5" t="s">
-        <v>21</v>
+      <c r="O60" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="P60" s="4" t="s">
         <v>27</v>
@@ -5334,31 +5337,31 @@
       <c r="T60" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="U60" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="V60" s="7" t="s">
-        <v>29</v>
+      <c r="U60" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="V60" s="5" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="61" spans="1:22">
       <c r="A61" s="4" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C61" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E61" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F61" s="5" t="s">
-        <v>21</v>
+      <c r="F61" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="G61" s="4" t="s">
         <v>27</v>
@@ -5375,17 +5378,17 @@
       <c r="K61" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="L61" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="M61" s="7" t="s">
-        <v>29</v>
+      <c r="L61" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="M61" s="5" t="s">
+        <v>22</v>
       </c>
       <c r="N61" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="O61" s="5" t="s">
-        <v>21</v>
+      <c r="O61" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="P61" s="4" t="s">
         <v>27</v>
@@ -5402,22 +5405,22 @@
       <c r="T61" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="U61" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="V61" s="7" t="s">
-        <v>29</v>
+      <c r="U61" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="V61" s="5" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="62" spans="1:22">
       <c r="A62" s="4" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D62" s="4" t="s">
         <v>65</v>
@@ -5479,10 +5482,10 @@
     </row>
     <row r="63" spans="1:22">
       <c r="A63" s="4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C63" s="4" t="s">
         <v>61</v>
@@ -5512,7 +5515,7 @@
         <v>61</v>
       </c>
       <c r="L63" s="6" t="s">
-        <v>85</v>
+        <v>117</v>
       </c>
       <c r="M63" s="6" t="s">
         <v>62</v>
@@ -5539,7 +5542,7 @@
         <v>61</v>
       </c>
       <c r="U63" s="6" t="s">
-        <v>85</v>
+        <v>117</v>
       </c>
       <c r="V63" s="6" t="s">
         <v>62</v>
@@ -5547,10 +5550,10 @@
     </row>
     <row r="64" spans="1:22">
       <c r="A64" s="4" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C64" s="4" t="s">
         <v>61</v>
@@ -5615,13 +5618,13 @@
     </row>
     <row r="65" spans="1:22">
       <c r="A65" s="4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D65" s="4" t="s">
         <v>80</v>
@@ -5683,13 +5686,13 @@
     </row>
     <row r="66" spans="1:22">
       <c r="A66" s="4" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D66" s="4" t="s">
         <v>80</v>
@@ -5751,16 +5754,16 @@
     </row>
     <row r="67" spans="1:22">
       <c r="A67" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E67" s="5" t="s">
         <v>20</v>
@@ -5784,11 +5787,11 @@
         <v>61</v>
       </c>
       <c r="L67" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="M67" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="M67" s="6" t="s">
-        <v>86</v>
-      </c>
       <c r="N67" s="5" t="s">
         <v>20</v>
       </c>
@@ -5811,25 +5814,25 @@
         <v>61</v>
       </c>
       <c r="U67" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="V67" s="6" t="s">
         <v>85</v>
-      </c>
-      <c r="V67" s="6" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="68" spans="1:22">
       <c r="A68" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D68" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="B68" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="C68" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D68" s="4" t="s">
-        <v>154</v>
-      </c>
       <c r="E68" s="5" t="s">
         <v>20</v>
       </c>
@@ -5852,11 +5855,11 @@
         <v>61</v>
       </c>
       <c r="L68" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="M68" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="M68" s="6" t="s">
-        <v>86</v>
-      </c>
       <c r="N68" s="5" t="s">
         <v>20</v>
       </c>
@@ -5879,24 +5882,24 @@
         <v>61</v>
       </c>
       <c r="U68" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="V68" s="6" t="s">
         <v>85</v>
-      </c>
-      <c r="V68" s="6" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="69" spans="1:22">
       <c r="A69" s="4" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C69" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D69" s="4" t="s">
         <v>42</v>
-      </c>
-      <c r="D69" s="4" t="s">
-        <v>43</v>
       </c>
       <c r="E69" s="5" t="s">
         <v>20</v>
@@ -5955,16 +5958,16 @@
     </row>
     <row r="70" spans="1:22">
       <c r="A70" s="4" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E70" s="5" t="s">
         <v>20</v>
@@ -6023,16 +6026,16 @@
     </row>
     <row r="71" spans="1:22">
       <c r="A71" s="4" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C71" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D71" s="4" t="s">
         <v>42</v>
-      </c>
-      <c r="D71" s="4" t="s">
-        <v>43</v>
       </c>
       <c r="E71" s="5" t="s">
         <v>20</v>
@@ -6091,16 +6094,16 @@
     </row>
     <row r="72" spans="1:22">
       <c r="A72" s="4" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C72" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D72" s="4" t="s">
         <v>42</v>
-      </c>
-      <c r="D72" s="4" t="s">
-        <v>43</v>
       </c>
       <c r="E72" s="4" t="s">
         <v>39</v>
@@ -6159,16 +6162,16 @@
     </row>
     <row r="73" spans="1:22">
       <c r="A73" s="4" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C73" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D73" s="4" t="s">
         <v>42</v>
-      </c>
-      <c r="D73" s="4" t="s">
-        <v>43</v>
       </c>
       <c r="E73" s="4" t="s">
         <v>39</v>
@@ -6227,16 +6230,16 @@
     </row>
     <row r="74" spans="1:22">
       <c r="A74" s="4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E74" s="5" t="s">
         <v>20</v>
@@ -6295,16 +6298,16 @@
     </row>
     <row r="75" spans="1:22">
       <c r="A75" s="4" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C75" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D75" s="4" t="s">
         <v>42</v>
-      </c>
-      <c r="D75" s="4" t="s">
-        <v>43</v>
       </c>
       <c r="E75" s="5" t="s">
         <v>20</v>
@@ -6363,10 +6366,10 @@
     </row>
     <row r="76" spans="1:22">
       <c r="A76" s="4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C76" s="4" t="s">
         <v>61</v>
@@ -6431,22 +6434,22 @@
     </row>
     <row r="77" spans="1:22">
       <c r="A77" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C77" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E77" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F77" s="5" t="s">
-        <v>21</v>
+      <c r="F77" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="G77" s="4" t="s">
         <v>27</v>
@@ -6467,13 +6470,13 @@
         <v>28</v>
       </c>
       <c r="M77" s="7" t="s">
-        <v>32</v>
+        <v>72</v>
       </c>
       <c r="N77" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="O77" s="5" t="s">
-        <v>21</v>
+      <c r="O77" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="P77" s="4" t="s">
         <v>27</v>
@@ -6494,21 +6497,21 @@
         <v>28</v>
       </c>
       <c r="V77" s="7" t="s">
-        <v>32</v>
+        <v>72</v>
       </c>
     </row>
     <row r="78" spans="1:22">
       <c r="A78" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C78" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E78" s="4" t="s">
         <v>39</v>
@@ -6562,27 +6565,27 @@
         <v>28</v>
       </c>
       <c r="V78" s="7" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
     </row>
     <row r="79" spans="1:22">
       <c r="A79" s="4" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C79" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E79" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F79" s="5" t="s">
-        <v>21</v>
+      <c r="F79" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="G79" s="4" t="s">
         <v>27</v>
@@ -6603,13 +6606,13 @@
         <v>28</v>
       </c>
       <c r="M79" s="7" t="s">
-        <v>32</v>
+        <v>72</v>
       </c>
       <c r="N79" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="O79" s="5" t="s">
-        <v>21</v>
+      <c r="O79" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="P79" s="4" t="s">
         <v>27</v>
@@ -6630,15 +6633,15 @@
         <v>28</v>
       </c>
       <c r="V79" s="7" t="s">
-        <v>32</v>
+        <v>72</v>
       </c>
     </row>
     <row r="80" spans="1:22">
       <c r="A80" s="4" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C80" s="4" t="s">
         <v>24</v>
@@ -6649,8 +6652,8 @@
       <c r="E80" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F80" s="5" t="s">
-        <v>21</v>
+      <c r="F80" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="G80" s="4" t="s">
         <v>27</v>
@@ -6671,13 +6674,13 @@
         <v>28</v>
       </c>
       <c r="M80" s="7" t="s">
-        <v>32</v>
+        <v>72</v>
       </c>
       <c r="N80" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="O80" s="5" t="s">
-        <v>21</v>
+      <c r="O80" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="P80" s="4" t="s">
         <v>27</v>
@@ -6698,15 +6701,15 @@
         <v>28</v>
       </c>
       <c r="V80" s="7" t="s">
-        <v>32</v>
+        <v>72</v>
       </c>
     </row>
     <row r="81" spans="1:22">
       <c r="A81" s="4" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C81" s="4" t="s">
         <v>61</v>
@@ -6771,10 +6774,10 @@
     </row>
     <row r="82" spans="1:22">
       <c r="A82" s="4" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C82" s="4" t="s">
         <v>61</v>
@@ -6839,10 +6842,10 @@
     </row>
     <row r="83" spans="1:22">
       <c r="A83" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C83" s="4" t="s">
         <v>61</v>
@@ -6907,10 +6910,10 @@
     </row>
     <row r="84" spans="1:22">
       <c r="A84" s="4" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C84" s="4" t="s">
         <v>61</v>
@@ -6975,7 +6978,7 @@
     </row>
     <row r="85" spans="1:22">
       <c r="A85" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B85" s="4" t="s">
         <v>64</v>
@@ -7043,10 +7046,10 @@
     </row>
     <row r="86" spans="1:22">
       <c r="A86" s="4" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C86" s="4" t="s">
         <v>61</v>
@@ -7111,10 +7114,10 @@
     </row>
     <row r="87" spans="1:22">
       <c r="A87" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C87" s="4" t="s">
         <v>61</v>
@@ -7179,10 +7182,10 @@
     </row>
     <row r="88" spans="1:22">
       <c r="A88" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C88" s="4" t="s">
         <v>61</v>
@@ -7247,10 +7250,10 @@
     </row>
     <row r="89" spans="1:22">
       <c r="A89" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C89" s="4" t="s">
         <v>61</v>
@@ -7315,10 +7318,10 @@
     </row>
     <row r="90" spans="1:22">
       <c r="A90" s="4" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C90" s="4" t="s">
         <v>61</v>
@@ -7383,10 +7386,10 @@
     </row>
     <row r="91" spans="1:22">
       <c r="A91" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C91" s="4" t="s">
         <v>61</v>
@@ -7451,16 +7454,16 @@
     </row>
     <row r="92" spans="1:22">
       <c r="A92" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E92" s="5" t="s">
         <v>20</v>
@@ -7484,11 +7487,11 @@
         <v>61</v>
       </c>
       <c r="L92" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="M92" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="M92" s="6" t="s">
-        <v>86</v>
-      </c>
       <c r="N92" s="5" t="s">
         <v>20</v>
       </c>
@@ -7511,18 +7514,18 @@
         <v>61</v>
       </c>
       <c r="U92" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="V92" s="6" t="s">
         <v>85</v>
-      </c>
-      <c r="V92" s="6" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="93" spans="1:22">
       <c r="A93" s="4" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C93" s="4" t="s">
         <v>61</v>
@@ -7552,7 +7555,7 @@
         <v>61</v>
       </c>
       <c r="L93" s="6" t="s">
-        <v>85</v>
+        <v>117</v>
       </c>
       <c r="M93" s="6" t="s">
         <v>62</v>
@@ -7579,7 +7582,7 @@
         <v>61</v>
       </c>
       <c r="U93" s="6" t="s">
-        <v>85</v>
+        <v>117</v>
       </c>
       <c r="V93" s="6" t="s">
         <v>62</v>
@@ -7587,16 +7590,16 @@
     </row>
     <row r="94" spans="1:22">
       <c r="A94" s="4" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E94" s="5" t="s">
         <v>20</v>
@@ -7655,10 +7658,10 @@
     </row>
     <row r="95" spans="1:22">
       <c r="A95" s="4" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C95" s="4" t="s">
         <v>61</v>
@@ -7723,7 +7726,7 @@
     </row>
     <row r="96" spans="1:22">
       <c r="A96" s="4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B96" s="4" t="s">
         <v>76</v>
@@ -7783,7 +7786,7 @@
         <v>61</v>
       </c>
       <c r="U96" s="6" t="s">
-        <v>85</v>
+        <v>117</v>
       </c>
       <c r="V96" s="6" t="s">
         <v>62</v>
@@ -7791,10 +7794,10 @@
     </row>
     <row r="97" spans="1:22">
       <c r="A97" s="4" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C97" s="4" t="s">
         <v>61</v>
@@ -7859,10 +7862,10 @@
     </row>
     <row r="98" spans="1:22">
       <c r="A98" s="4" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C98" s="4" t="s">
         <v>61</v>
@@ -7919,7 +7922,7 @@
         <v>61</v>
       </c>
       <c r="U98" s="6" t="s">
-        <v>85</v>
+        <v>117</v>
       </c>
       <c r="V98" s="6" t="s">
         <v>62</v>
@@ -7927,10 +7930,10 @@
     </row>
     <row r="99" spans="1:22">
       <c r="A99" s="4" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C99" s="4" t="s">
         <v>61</v>
@@ -7987,7 +7990,7 @@
         <v>61</v>
       </c>
       <c r="U99" s="6" t="s">
-        <v>85</v>
+        <v>117</v>
       </c>
       <c r="V99" s="6" t="s">
         <v>62</v>
@@ -7995,16 +7998,16 @@
     </row>
     <row r="100" spans="1:22">
       <c r="A100" s="4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C100" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D100" s="4" t="s">
         <v>42</v>
-      </c>
-      <c r="D100" s="4" t="s">
-        <v>43</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>26</v>
@@ -8031,7 +8034,7 @@
         <v>28</v>
       </c>
       <c r="M100" s="7" t="s">
-        <v>29</v>
+        <v>120</v>
       </c>
       <c r="N100" s="6" t="s">
         <v>26</v>
@@ -8058,15 +8061,15 @@
         <v>28</v>
       </c>
       <c r="V100" s="7" t="s">
-        <v>29</v>
+        <v>120</v>
       </c>
     </row>
     <row r="101" spans="1:22">
       <c r="A101" s="4" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C101" s="4" t="s">
         <v>61</v>
@@ -8131,10 +8134,10 @@
     </row>
     <row r="102" spans="1:22">
       <c r="A102" s="4" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C102" s="4" t="s">
         <v>61</v>
@@ -8199,10 +8202,10 @@
     </row>
     <row r="103" spans="1:22">
       <c r="A103" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C103" s="4" t="s">
         <v>61</v>
@@ -8267,13 +8270,13 @@
     </row>
     <row r="104" spans="1:22">
       <c r="A104" s="4" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C104" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D104" s="4" t="s">
         <v>65</v>
@@ -8335,10 +8338,10 @@
     </row>
     <row r="105" spans="1:22">
       <c r="A105" s="4" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C105" s="4" t="s">
         <v>61</v>
@@ -8403,10 +8406,10 @@
     </row>
     <row r="106" spans="1:22">
       <c r="A106" s="4" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B106" s="4" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C106" s="4" t="s">
         <v>61</v>
@@ -8471,10 +8474,10 @@
     </row>
     <row r="107" spans="1:22">
       <c r="A107" s="4" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C107" s="4" t="s">
         <v>61</v>
@@ -8539,10 +8542,10 @@
     </row>
     <row r="108" spans="1:22">
       <c r="A108" s="4" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C108" s="4" t="s">
         <v>61</v>
@@ -8607,10 +8610,10 @@
     </row>
     <row r="109" spans="1:22">
       <c r="A109" s="4" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C109" s="4" t="s">
         <v>61</v>
@@ -8675,16 +8678,16 @@
     </row>
     <row r="110" spans="1:22">
       <c r="A110" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C110" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D110" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E110" s="5" t="s">
         <v>20</v>
@@ -8743,16 +8746,16 @@
     </row>
     <row r="111" spans="1:22">
       <c r="A111" s="4" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C111" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D111" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E111" s="5" t="s">
         <v>20</v>
@@ -8811,16 +8814,16 @@
     </row>
     <row r="112" spans="1:22">
       <c r="A112" s="4" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C112" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D112" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E112" s="5" t="s">
         <v>20</v>
@@ -8879,16 +8882,16 @@
     </row>
     <row r="113" spans="1:22">
       <c r="A113" s="4" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C113" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D113" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E113" s="5" t="s">
         <v>20</v>
@@ -8947,16 +8950,16 @@
     </row>
     <row r="114" spans="1:22">
       <c r="A114" s="4" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C114" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D114" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E114" s="5" t="s">
         <v>20</v>
@@ -9015,13 +9018,13 @@
     </row>
     <row r="115" spans="1:22">
       <c r="A115" s="4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C115" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D115" s="4" t="s">
         <v>77</v>
@@ -9083,13 +9086,13 @@
     </row>
     <row r="116" spans="1:22">
       <c r="A116" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C116" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D116" s="4" t="s">
         <v>65</v>
@@ -9151,13 +9154,13 @@
     </row>
     <row r="117" spans="1:22">
       <c r="A117" s="4" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C117" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D117" s="4" t="s">
         <v>68</v>
@@ -9219,16 +9222,16 @@
     </row>
     <row r="118" spans="1:22">
       <c r="A118" s="4" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C118" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D118" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E118" s="5" t="s">
         <v>20</v>
@@ -9287,13 +9290,13 @@
     </row>
     <row r="119" spans="1:22">
       <c r="A119" s="4" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C119" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D119" s="4" t="s">
         <v>68</v>
@@ -9355,16 +9358,16 @@
     </row>
     <row r="120" spans="1:22">
       <c r="A120" s="4" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C120" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D120" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E120" s="5" t="s">
         <v>20</v>
@@ -9423,10 +9426,10 @@
     </row>
     <row r="121" spans="1:22">
       <c r="A121" s="4" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C121" s="4" t="s">
         <v>61</v>
@@ -9491,10 +9494,10 @@
     </row>
     <row r="122" spans="1:22">
       <c r="A122" s="4" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C122" s="4" t="s">
         <v>61</v>
@@ -9559,10 +9562,10 @@
     </row>
     <row r="123" spans="1:22">
       <c r="A123" s="4" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C123" s="4" t="s">
         <v>61</v>
@@ -9627,16 +9630,16 @@
     </row>
     <row r="124" spans="1:22">
       <c r="A124" s="4" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C124" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D124" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E124" s="4" t="s">
         <v>39</v>
@@ -9695,16 +9698,16 @@
     </row>
     <row r="125" spans="1:22">
       <c r="A125" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B125" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="B125" s="4" t="s">
-        <v>265</v>
-      </c>
       <c r="C125" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D125" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E125" s="4" t="s">
         <v>39</v>
@@ -9763,16 +9766,16 @@
     </row>
     <row r="126" spans="1:22">
       <c r="A126" s="4" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C126" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D126" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E126" s="4" t="s">
         <v>39</v>
@@ -9826,21 +9829,21 @@
         <v>28</v>
       </c>
       <c r="V126" s="7" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
     </row>
     <row r="127" spans="1:22">
       <c r="A127" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="B127" s="4" t="s">
         <v>269</v>
-      </c>
-      <c r="B127" s="4" t="s">
-        <v>268</v>
       </c>
       <c r="C127" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D127" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E127" s="4" t="s">
         <v>39</v>
@@ -9894,27 +9897,27 @@
         <v>28</v>
       </c>
       <c r="V127" s="7" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
     </row>
     <row r="128" spans="1:22">
       <c r="A128" s="4" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C128" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D128" s="4" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E128" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F128" s="5" t="s">
-        <v>21</v>
+      <c r="F128" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="G128" s="4" t="s">
         <v>27</v>
@@ -9935,13 +9938,13 @@
         <v>28</v>
       </c>
       <c r="M128" s="7" t="s">
-        <v>32</v>
+        <v>72</v>
       </c>
       <c r="N128" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="O128" s="5" t="s">
-        <v>21</v>
+      <c r="O128" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="P128" s="4" t="s">
         <v>27</v>
@@ -9962,21 +9965,21 @@
         <v>28</v>
       </c>
       <c r="V128" s="7" t="s">
-        <v>32</v>
+        <v>72</v>
       </c>
     </row>
     <row r="129" spans="1:22">
       <c r="A129" s="4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C129" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D129" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E129" s="4" t="s">
         <v>39</v>
@@ -10030,21 +10033,21 @@
         <v>28</v>
       </c>
       <c r="V129" s="7" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
     </row>
     <row r="130" spans="1:22">
       <c r="A130" s="4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C130" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D130" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E130" s="4" t="s">
         <v>39</v>
@@ -10098,15 +10101,15 @@
         <v>28</v>
       </c>
       <c r="V130" s="7" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
     </row>
     <row r="131" spans="1:22">
       <c r="A131" s="4" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C131" s="4" t="s">
         <v>18</v>
@@ -10171,10 +10174,10 @@
     </row>
     <row r="132" spans="1:22">
       <c r="A132" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="B132" s="4" t="s">
         <v>276</v>
-      </c>
-      <c r="B132" s="4" t="s">
-        <v>275</v>
       </c>
       <c r="C132" s="4" t="s">
         <v>61</v>
@@ -10239,10 +10242,10 @@
     </row>
     <row r="133" spans="1:22">
       <c r="A133" s="4" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C133" s="4" t="s">
         <v>61</v>
@@ -10307,10 +10310,10 @@
     </row>
     <row r="134" spans="1:22">
       <c r="A134" s="4" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C134" s="4" t="s">
         <v>61</v>
@@ -10375,10 +10378,10 @@
     </row>
     <row r="135" spans="1:22">
       <c r="A135" s="4" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C135" s="4" t="s">
         <v>61</v>
@@ -10443,10 +10446,10 @@
     </row>
     <row r="136" spans="1:22">
       <c r="A136" s="4" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C136" s="4" t="s">
         <v>61</v>
@@ -10511,10 +10514,10 @@
     </row>
     <row r="137" spans="1:22">
       <c r="A137" s="4" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C137" s="4" t="s">
         <v>61</v>
@@ -10579,10 +10582,10 @@
     </row>
     <row r="138" spans="1:22">
       <c r="A138" s="4" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C138" s="4" t="s">
         <v>61</v>
@@ -10647,10 +10650,10 @@
     </row>
     <row r="139" spans="1:22">
       <c r="A139" s="4" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C139" s="4" t="s">
         <v>61</v>
@@ -10715,10 +10718,10 @@
     </row>
     <row r="140" spans="1:22">
       <c r="A140" s="4" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C140" s="4" t="s">
         <v>61</v>
@@ -10801,7 +10804,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -10810,19 +10813,19 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>22</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -10833,10 +10836,10 @@
         <v>137</v>
       </c>
       <c r="C3" s="5">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D3" s="7">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E3" s="6">
         <v>47</v>
@@ -10850,10 +10853,10 @@
         <v>137</v>
       </c>
       <c r="C4" s="5">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D4" s="7">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E4" s="6">
         <v>47</v>

</xml_diff>